<commit_message>
Update New Relic market reports - 2026-10-14 01:30:38
</commit_message>
<xml_diff>
--- a/output/japan.xlsx
+++ b/output/japan.xlsx
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>340</v>
+        <v>351</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="D35" s="6" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>